<commit_message>
variabili per Tabella 1
</commit_message>
<xml_diff>
--- a/i_test/test_D3_coorte_con_caratterizzazione/dia_angi.xlsx
+++ b/i_test/test_D3_coorte_con_caratterizzazione/dia_angi.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -28,6 +28,12 @@
     <t xml:space="preserve">DATE</t>
   </si>
   <si>
+    <t xml:space="preserve">Table_cdm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ord</t>
+  </si>
+  <si>
     <t xml:space="preserve">P01</t>
   </si>
   <si>
@@ -35,6 +41,12 @@
   </si>
   <si>
     <t xml:space="preserve">P03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P04</t>
   </si>
 </sst>
 </file>
@@ -148,7 +160,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -158,10 +170,16 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>-730</v>
@@ -169,18 +187,35 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>2500</v>
       </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>2500</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2500</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>